<commit_message>
Changes for data csv & Feature data load logic
</commit_message>
<xml_diff>
--- a/src/helper/util/test-data/testData.xlsx
+++ b/src/helper/util/test-data/testData.xlsx
@@ -37,7 +37,7 @@
     <t>Apple@1234567</t>
   </si>
   <si>
-    <t>Login-InValid</t>
+    <t>staging_Login-InValid</t>
   </si>
 </sst>
 </file>
@@ -55,7 +55,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -432,7 +432,7 @@
     <col min="4" max="4" style="6" width="15.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>